<commit_message>
Atualizei tabela de referência.
</commit_message>
<xml_diff>
--- a/refs/entregavel_tabela.xlsx
+++ b/refs/entregavel_tabela.xlsx
@@ -9,14 +9,11 @@
   </sheets>
   <definedNames/>
   <calcPr/>
-  <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId8"/>
-  </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
   <si>
     <t>nome_ator</t>
   </si>
@@ -24,82 +21,91 @@
     <t>nacionalidade</t>
   </si>
   <si>
+    <t>grupo_geral_nacionalidade</t>
+  </si>
+  <si>
+    <t>grupo_especifico_nacionalidade</t>
+  </si>
+  <si>
+    <t>filme_indicado</t>
+  </si>
+  <si>
+    <t>ano_filme</t>
+  </si>
+  <si>
+    <t>numero_cerimonia</t>
+  </si>
+  <si>
+    <t>ano_cerimonia</t>
+  </si>
+  <si>
+    <t>url_ator</t>
+  </si>
+  <si>
+    <t>url_filme</t>
+  </si>
+  <si>
+    <t>url_cerimonia</t>
+  </si>
+  <si>
+    <t>Adrien Brody</t>
+  </si>
+  <si>
+    <t>EUA</t>
+  </si>
+  <si>
+    <t>The Brutalist</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Adrien_Brody</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/The_Brutalist</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/97th_Academy_Awards</t>
+  </si>
+  <si>
+    <t>Cillian Murphy</t>
+  </si>
+  <si>
+    <t>Irlanda</t>
+  </si>
+  <si>
+    <t>Europeu</t>
+  </si>
+  <si>
+    <t>Oppenheimer</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Cillian_Murphy</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Oppenheimer_(film)</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/96th_Academy_Awards</t>
+  </si>
+  <si>
+    <t>Brendan Fraser</t>
+  </si>
+  <si>
+    <t>The Whale</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Brendan_Fraser</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/The_Whale_(2022_film)</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/95th_Academy_Awards</t>
+  </si>
+  <si>
     <t>grupo_nacionalidade</t>
   </si>
   <si>
-    <t>filme_indicado</t>
-  </si>
-  <si>
-    <t>numero_cerimonia</t>
-  </si>
-  <si>
-    <t>ano_cerimonia</t>
-  </si>
-  <si>
-    <t>url_ator</t>
-  </si>
-  <si>
-    <t>url_filme</t>
-  </si>
-  <si>
-    <t>url_cerimonia</t>
-  </si>
-  <si>
-    <t>Adrien Brody</t>
-  </si>
-  <si>
-    <t>EUA</t>
-  </si>
-  <si>
-    <t>The Brutalist</t>
-  </si>
-  <si>
-    <t>https://en.wikipedia.org/wiki/Adrien_Brody</t>
-  </si>
-  <si>
-    <t>https://en.wikipedia.org/wiki/The_Brutalist</t>
-  </si>
-  <si>
-    <t>https://en.wikipedia.org/wiki/97th_Academy_Awards</t>
-  </si>
-  <si>
-    <t>Cillian Murphy</t>
-  </si>
-  <si>
-    <t>Irlanda</t>
-  </si>
-  <si>
-    <t>Oppenheimer</t>
-  </si>
-  <si>
-    <t>https://en.wikipedia.org/wiki/Cillian_Murphy</t>
-  </si>
-  <si>
-    <t>https://en.wikipedia.org/wiki/Oppenheimer_(film)</t>
-  </si>
-  <si>
-    <t>https://en.wikipedia.org/wiki/96th_Academy_Awards</t>
-  </si>
-  <si>
-    <t>Brendan Fraser</t>
-  </si>
-  <si>
-    <t>The Whale</t>
-  </si>
-  <si>
-    <t>https://en.wikipedia.org/wiki/Brendan_Fraser</t>
-  </si>
-  <si>
-    <t>https://en.wikipedia.org/wiki/The_Whale_(2022_film)</t>
-  </si>
-  <si>
-    <t>https://en.wikipedia.org/wiki/95th_Academy_Awards</t>
-  </si>
-  <si>
-    <t>COUNTA de nome_ator</t>
-  </si>
-  <si>
-    <t>Estrangeiro</t>
+    <t>vencedores</t>
   </si>
 </sst>
 </file>
@@ -213,7 +219,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>agregada!$B$1</c:f>
+              <c:f>agregada!$B$2</c:f>
             </c:strRef>
           </c:tx>
           <c:dPt>
@@ -226,11 +232,6 @@
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="6AA84F"/>
-              </a:solidFill>
-            </c:spPr>
           </c:dPt>
           <c:dLbls>
             <c:showLegendKey val="0"/>
@@ -243,12 +244,12 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>agregada!$A$2:$A$3</c:f>
+              <c:f>agregada!$A$3:$A$4</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>agregada!$B$2:$B$3</c:f>
+              <c:f>agregada!$B$3:$B$4</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -327,147 +328,6 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" invalid="1" refreshOnLoad="1">
-  <cacheSource type="worksheet">
-    <worksheetSource ref="A1:I3" sheet="crua"/>
-  </cacheSource>
-  <cacheFields>
-    <cacheField name="nome_ator" numFmtId="0">
-      <sharedItems>
-        <s v="Adrien Brody"/>
-        <s v="Cillian Murphy"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="nacionalidade" numFmtId="0">
-      <sharedItems>
-        <s v="EUA"/>
-        <s v="Irlanda"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="grupo_nacionalidade" numFmtId="0">
-      <sharedItems>
-        <s v="EUA"/>
-        <s v="Estrangeiro"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="filme_indicado" numFmtId="0">
-      <sharedItems>
-        <s v="The Brutalist"/>
-        <s v="Oppenheimer"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="numero_cerimonia" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
-        <n v="97.0"/>
-        <n v="96.0"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="ano_cerimonia" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
-        <n v="2025.0"/>
-        <n v="2024.0"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="url_ator" numFmtId="0">
-      <sharedItems>
-        <s v="https://en.wikipedia.org/wiki/Adrien_Brody"/>
-        <s v="https://en.wikipedia.org/wiki/Cillian_Murphy"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="url_filme" numFmtId="0">
-      <sharedItems>
-        <s v="https://en.wikipedia.org/wiki/The_Brutalist"/>
-        <s v="https://en.wikipedia.org/wiki/Oppenheimer_(film)"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="url_cerimonia" numFmtId="0">
-      <sharedItems>
-        <s v="https://en.wikipedia.org/wiki/97th_Academy_Awards"/>
-        <s v="https://en.wikipedia.org/wiki/96th_Academy_Awards"/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="agregada" cacheId="0" dataCaption="" rowGrandTotals="0" compact="0" compactData="0">
-  <location ref="A1:B3" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields>
-    <pivotField name="nome_ator" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="nacionalidade" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="grupo_nacionalidade" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items>
-        <item x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="filme_indicado" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="numero_cerimonia" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="ano_cerimonia" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="url_ator" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="url_filme" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="url_cerimonia" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields>
-    <field x="2"/>
-  </rowFields>
-  <dataFields>
-    <dataField name="COUNTA of nome_ator" fld="0" subtotal="count" baseField="0"/>
-  </dataFields>
-</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -672,10 +532,10 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="14.0"/>
-    <col customWidth="1" min="4" max="4" width="12.63"/>
-    <col customWidth="1" min="7" max="7" width="33.75"/>
-    <col customWidth="1" min="8" max="8" width="39.5"/>
-    <col customWidth="1" min="9" max="9" width="39.38"/>
+    <col customWidth="1" min="5" max="5" width="12.63"/>
+    <col customWidth="1" min="9" max="9" width="33.75"/>
+    <col customWidth="1" min="10" max="10" width="39.5"/>
+    <col customWidth="1" min="11" max="11" width="39.38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -706,6 +566,177 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+      <c r="Z1" s="2"/>
+      <c r="AA1" s="2"/>
+      <c r="AB1" s="2"/>
+      <c r="AC1" s="2"/>
+      <c r="AD1" s="2"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="3" t="str">
+        <f t="shared" ref="C2:C4" si="1">IF(B2="EUA", "EUA","Estrangeiro")</f>
+        <v>EUA</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3">
+        <v>2024.0</v>
+      </c>
+      <c r="G2" s="3">
+        <v>97.0</v>
+      </c>
+      <c r="H2" s="3">
+        <v>2025.0</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>Estrangeiro</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="3">
+        <v>2023.0</v>
+      </c>
+      <c r="G3" s="3">
+        <v>96.0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>2024.0</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>EUA</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="3">
+        <v>2022.0</v>
+      </c>
+      <c r="G4" s="3">
+        <v>95.0</v>
+      </c>
+      <c r="H4" s="3">
+        <v>2023.0</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="I2"/>
+    <hyperlink r:id="rId2" ref="J2"/>
+    <hyperlink r:id="rId3" ref="K2"/>
+    <hyperlink r:id="rId4" ref="I3"/>
+    <hyperlink r:id="rId5" ref="J3"/>
+    <hyperlink r:id="rId6" ref="K3"/>
+    <hyperlink r:id="rId7" ref="I4"/>
+    <hyperlink r:id="rId8" ref="J4"/>
+    <hyperlink r:id="rId9" ref="K4"/>
+  </hyperlinks>
+  <drawing r:id="rId10"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
@@ -723,127 +754,28 @@
       <c r="X1" s="2"/>
       <c r="Y1" s="2"/>
       <c r="Z1" s="2"/>
-      <c r="AA1" s="2"/>
-      <c r="AB1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="3" t="str">
-        <f t="shared" ref="C2:C4" si="1">IF(B2="EUA", "EUA","Estrangeiro")</f>
+      <c r="A2" s="6" t="str">
+        <f t="array" ref="A2:A3">UNIQUE(crua!$B$2:$B$4)</f>
         <v>EUA</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="3">
-        <v>97.0</v>
-      </c>
-      <c r="F2" s="3">
-        <v>2025.0</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>14</v>
+      <c r="B2" s="6">
+        <f>COUNTIF(crua!$B$1:$B$4, A2)</f>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Estrangeiro</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="3">
-        <v>96.0</v>
-      </c>
-      <c r="F3" s="3">
-        <v>2024.0</v>
-      </c>
-      <c r="G3" s="4" t="s">
+      <c r="A3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>EUA</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="3">
-        <v>95.0</v>
-      </c>
-      <c r="F4" s="3">
-        <v>2023.0</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>25</v>
+      <c r="B3" s="6">
+        <f>COUNTIF(crua!$B$1:$B$4, A3)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="G2"/>
-    <hyperlink r:id="rId2" ref="H2"/>
-    <hyperlink r:id="rId3" ref="I2"/>
-    <hyperlink r:id="rId4" ref="G3"/>
-    <hyperlink r:id="rId5" ref="H3"/>
-    <hyperlink r:id="rId6" ref="I3"/>
-    <hyperlink r:id="rId7" ref="G4"/>
-    <hyperlink r:id="rId8" ref="H4"/>
-    <hyperlink r:id="rId9" ref="I4"/>
-  </hyperlinks>
-  <drawing r:id="rId10"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-  </sheetData>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>